<commit_message>
Se finaliza MAestro de Tolerancias
</commit_message>
<xml_diff>
--- a/documentos/RQM Aprobacion Ajustes OC/2028-08-29 Costos Aprobacion_OC.xlsx
+++ b/documentos/RQM Aprobacion Ajustes OC/2028-08-29 Costos Aprobacion_OC.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Personal\Promos\Nuevos Requerimientos\2026-08-29 Requerimiento Aprobacion Ajustes OC Confirmadas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Personal\Promos\Repos\Aldebaran.Web\documentos\RQM Aprobacion Ajustes OC\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="6855" windowWidth="28800" windowHeight="11805" tabRatio="680" firstSheet="1" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="7305" windowWidth="28800" windowHeight="11805" tabRatio="680" firstSheet="1" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Identificación e Instrucciones" sheetId="6" r:id="rId1"/>
@@ -248,7 +248,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="180">
   <si>
     <t>Datos del proyecto</t>
   </si>
@@ -906,6 +906,9 @@
   </si>
   <si>
     <t>Entrega Final</t>
+  </si>
+  <si>
+    <t>Total Esfuerzo Basado en 8 Horas</t>
   </si>
 </sst>
 </file>
@@ -1047,7 +1050,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1147,6 +1150,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1643,7 +1652,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
@@ -1813,12 +1822,6 @@
     <xf numFmtId="3" fontId="1" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -1829,22 +1832,41 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="13" fillId="9" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1888,35 +1910,22 @@
     <xf numFmtId="0" fontId="15" fillId="15" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="13" fillId="9" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="10" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1940,6 +1949,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2317,87 +2332,87 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="122" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="123"/>
+      <c r="A1" s="120" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="121"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="119" t="s">
+      <c r="A2" s="122" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="120"/>
-      <c r="C2" s="121"/>
-      <c r="D2" s="121"/>
-      <c r="E2" s="121"/>
-      <c r="F2" s="121"/>
-      <c r="G2" s="121"/>
+      <c r="B2" s="123"/>
+      <c r="C2" s="119"/>
+      <c r="D2" s="119"/>
+      <c r="E2" s="119"/>
+      <c r="F2" s="119"/>
+      <c r="G2" s="119"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="119" t="s">
+      <c r="A3" s="122" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="120"/>
-      <c r="C3" s="121"/>
-      <c r="D3" s="121"/>
-      <c r="E3" s="121"/>
-      <c r="F3" s="121"/>
-      <c r="G3" s="121"/>
+      <c r="B3" s="123"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="119"/>
+      <c r="F3" s="119"/>
+      <c r="G3" s="119"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="119" t="s">
+      <c r="A4" s="122" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="120"/>
-      <c r="C4" s="121"/>
-      <c r="D4" s="121"/>
-      <c r="E4" s="121"/>
-      <c r="F4" s="121"/>
-      <c r="G4" s="121"/>
+      <c r="B4" s="123"/>
+      <c r="C4" s="119"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="119"/>
+      <c r="F4" s="119"/>
+      <c r="G4" s="119"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="119" t="s">
+      <c r="A5" s="122" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="120"/>
-      <c r="C5" s="121"/>
-      <c r="D5" s="121"/>
-      <c r="E5" s="121"/>
-      <c r="F5" s="121"/>
-      <c r="G5" s="121"/>
+      <c r="B5" s="123"/>
+      <c r="C5" s="119"/>
+      <c r="D5" s="119"/>
+      <c r="E5" s="119"/>
+      <c r="F5" s="119"/>
+      <c r="G5" s="119"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="97"/>
-      <c r="C6" s="121"/>
-      <c r="D6" s="121"/>
-      <c r="E6" s="121"/>
-      <c r="F6" s="121"/>
-      <c r="G6" s="121"/>
+      <c r="C6" s="119"/>
+      <c r="D6" s="119"/>
+      <c r="E6" s="119"/>
+      <c r="F6" s="119"/>
+      <c r="G6" s="119"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="119" t="s">
+      <c r="A7" s="122" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="120"/>
-      <c r="C7" s="121"/>
-      <c r="D7" s="121"/>
-      <c r="E7" s="121"/>
-      <c r="F7" s="121"/>
-      <c r="G7" s="121"/>
+      <c r="B7" s="123"/>
+      <c r="C7" s="119"/>
+      <c r="D7" s="119"/>
+      <c r="E7" s="119"/>
+      <c r="F7" s="119"/>
+      <c r="G7" s="119"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="122" t="s">
+      <c r="A8" s="120" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="123"/>
-      <c r="C8" s="121"/>
-      <c r="D8" s="121"/>
-      <c r="E8" s="121"/>
-      <c r="F8" s="121"/>
-      <c r="G8" s="121"/>
+      <c r="B8" s="121"/>
+      <c r="C8" s="119"/>
+      <c r="D8" s="119"/>
+      <c r="E8" s="119"/>
+      <c r="F8" s="119"/>
+      <c r="G8" s="119"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="55"/>
@@ -2546,6 +2561,11 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="14">
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C6:G6"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="C5:G5"/>
@@ -2555,11 +2575,6 @@
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C4:G4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C6:G6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2594,15 +2609,15 @@
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A2" s="143" t="s">
+      <c r="A2" s="133" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="143"/>
-      <c r="C2" s="143"/>
-      <c r="D2" s="143"/>
-      <c r="E2" s="143"/>
+      <c r="B2" s="133"/>
+      <c r="C2" s="133"/>
+      <c r="D2" s="133"/>
+      <c r="E2" s="133"/>
       <c r="F2" s="118">
-        <v>9.5</v>
+        <v>2</v>
       </c>
       <c r="H2" s="98" t="s">
         <v>31</v>
@@ -2614,142 +2629,153 @@
       <c r="M2" s="100"/>
       <c r="N2" s="69">
         <f>CEILING(F2*(8/F4),1)</f>
-        <v>19</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="P2" s="160" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q2" s="160"/>
       <c r="AA2" s="13" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A3" s="143" t="s">
+      <c r="A3" s="133" t="s">
         <v>163</v>
       </c>
-      <c r="B3" s="143"/>
-      <c r="C3" s="143"/>
-      <c r="D3" s="143"/>
-      <c r="E3" s="143"/>
+      <c r="B3" s="133"/>
+      <c r="C3" s="133"/>
+      <c r="D3" s="133"/>
+      <c r="E3" s="133"/>
       <c r="F3" s="63">
         <v>1</v>
       </c>
-      <c r="H3" s="146" t="s">
+      <c r="H3" s="126" t="s">
         <v>32</v>
       </c>
-      <c r="I3" s="147"/>
-      <c r="J3" s="147"/>
-      <c r="K3" s="147"/>
-      <c r="L3" s="147"/>
-      <c r="M3" s="148"/>
+      <c r="I3" s="127"/>
+      <c r="J3" s="127"/>
+      <c r="K3" s="127"/>
+      <c r="L3" s="127"/>
+      <c r="M3" s="128"/>
       <c r="N3" s="67">
         <f>CEILING(N2/F3,1)</f>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A4" s="143" t="s">
+        <v>4</v>
+      </c>
+      <c r="P3" s="160"/>
+      <c r="Q3" s="160"/>
+    </row>
+    <row r="4" spans="1:27" ht="18" x14ac:dyDescent="0.25">
+      <c r="A4" s="133" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="143"/>
-      <c r="C4" s="143"/>
-      <c r="D4" s="143"/>
-      <c r="E4" s="143"/>
+      <c r="B4" s="133"/>
+      <c r="C4" s="133"/>
+      <c r="D4" s="133"/>
+      <c r="E4" s="133"/>
       <c r="F4" s="63">
         <v>4</v>
       </c>
-      <c r="H4" s="149" t="s">
+      <c r="H4" s="129" t="s">
         <v>34</v>
       </c>
-      <c r="I4" s="150"/>
-      <c r="J4" s="150"/>
-      <c r="K4" s="150"/>
-      <c r="L4" s="150"/>
-      <c r="M4" s="151"/>
+      <c r="I4" s="130"/>
+      <c r="J4" s="130"/>
+      <c r="K4" s="130"/>
+      <c r="L4" s="130"/>
+      <c r="M4" s="131"/>
       <c r="N4" s="67">
         <f>CEILING((N3/F7)+F8,1)</f>
-        <v>19</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="P4" s="161">
+        <f>F2+((F5+F6+F8)*F7)+F11+F12+F13+F14+F15</f>
+        <v>4.5</v>
+      </c>
+      <c r="Q4" s="161"/>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A5" s="143" t="s">
+      <c r="A5" s="133" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="143"/>
-      <c r="C5" s="143"/>
-      <c r="D5" s="143"/>
-      <c r="E5" s="143"/>
+      <c r="B5" s="133"/>
+      <c r="C5" s="133"/>
+      <c r="D5" s="133"/>
+      <c r="E5" s="133"/>
       <c r="F5" s="63">
         <v>0</v>
       </c>
-      <c r="H5" s="149" t="str">
+      <c r="H5" s="129" t="str">
         <f>IF(F7&gt;1, CONCATENATE("Duración de desarrollo de los Iteración 2 a ",F7,":"),"Duración Iteración 2 en adelante")</f>
         <v>Duración Iteración 2 en adelante</v>
       </c>
-      <c r="I5" s="150"/>
-      <c r="J5" s="150"/>
-      <c r="K5" s="150"/>
-      <c r="L5" s="150"/>
-      <c r="M5" s="151"/>
+      <c r="I5" s="130"/>
+      <c r="J5" s="130"/>
+      <c r="K5" s="130"/>
+      <c r="L5" s="130"/>
+      <c r="M5" s="131"/>
       <c r="N5" s="67">
         <f>IF(F7&gt;1,CEILING( (N3/F7),1),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A6" s="143" t="s">
+      <c r="A6" s="133" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="143"/>
-      <c r="C6" s="143"/>
-      <c r="D6" s="143"/>
-      <c r="E6" s="143"/>
+      <c r="B6" s="133"/>
+      <c r="C6" s="133"/>
+      <c r="D6" s="133"/>
+      <c r="E6" s="133"/>
       <c r="F6" s="63">
         <v>0</v>
       </c>
-      <c r="H6" s="149" t="s">
+      <c r="H6" s="129" t="s">
         <v>37</v>
       </c>
-      <c r="I6" s="150"/>
-      <c r="J6" s="150"/>
-      <c r="K6" s="150"/>
-      <c r="L6" s="150"/>
-      <c r="M6" s="151"/>
+      <c r="I6" s="130"/>
+      <c r="J6" s="130"/>
+      <c r="K6" s="130"/>
+      <c r="L6" s="130"/>
+      <c r="M6" s="131"/>
       <c r="N6" s="67">
         <f>CEILING( N4+F5+F6,1)</f>
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="143" t="s">
+      <c r="A7" s="133" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="143"/>
-      <c r="C7" s="143"/>
-      <c r="D7" s="143"/>
-      <c r="E7" s="143"/>
+      <c r="B7" s="133"/>
+      <c r="C7" s="133"/>
+      <c r="D7" s="133"/>
+      <c r="E7" s="133"/>
       <c r="F7" s="63">
         <v>1</v>
       </c>
-      <c r="H7" s="149" t="str">
+      <c r="H7" s="129" t="str">
         <f>IF(F7&gt;1, CONCATENATE("Duración total de los Iteración 2 a ",F7," (incluye planeación y presentación):"),"Duración Iteración 2 en adelante  (incluye planeación y presentación)")</f>
         <v>Duración Iteración 2 en adelante  (incluye planeación y presentación)</v>
       </c>
-      <c r="I7" s="150"/>
-      <c r="J7" s="150"/>
-      <c r="K7" s="150"/>
-      <c r="L7" s="150"/>
-      <c r="M7" s="152"/>
+      <c r="I7" s="130"/>
+      <c r="J7" s="130"/>
+      <c r="K7" s="130"/>
+      <c r="L7" s="130"/>
+      <c r="M7" s="132"/>
       <c r="N7" s="70">
         <f>IF(F7&gt;1, CEILING( N5+F5+F6,1),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:27" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="143" t="s">
+      <c r="A8" s="133" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="143"/>
-      <c r="C8" s="143"/>
-      <c r="D8" s="143"/>
-      <c r="E8" s="143"/>
+      <c r="B8" s="133"/>
+      <c r="C8" s="133"/>
+      <c r="D8" s="133"/>
+      <c r="E8" s="133"/>
       <c r="F8" s="63">
         <v>0</v>
       </c>
@@ -2759,7 +2785,7 @@
       <c r="M8" s="71"/>
       <c r="N8" s="72">
         <f>((N6+(N7*(F7-1))))</f>
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.2">
@@ -2786,89 +2812,89 @@
       <c r="J10" s="109"/>
     </row>
     <row r="11" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="143" t="s">
+      <c r="A11" s="133" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="143"/>
-      <c r="C11" s="143"/>
-      <c r="D11" s="143"/>
-      <c r="E11" s="143"/>
+      <c r="B11" s="133"/>
+      <c r="C11" s="133"/>
+      <c r="D11" s="133"/>
+      <c r="E11" s="133"/>
       <c r="F11" s="63">
         <v>0.5</v>
       </c>
-      <c r="H11" s="144" t="str">
+      <c r="H11" s="124" t="str">
         <f>CONCATENATE(N8+F12+F13+F14+F15+F11, " días")</f>
-        <v>22 días</v>
-      </c>
-      <c r="I11" s="144"/>
-      <c r="J11" s="144"/>
+        <v>6.5 días</v>
+      </c>
+      <c r="I11" s="124"/>
+      <c r="J11" s="124"/>
       <c r="K11" s="68" t="s">
         <v>43</v>
       </c>
       <c r="L11" s="68"/>
     </row>
     <row r="12" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="143" t="s">
+      <c r="A12" s="133" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="143"/>
-      <c r="C12" s="143"/>
-      <c r="D12" s="143"/>
-      <c r="E12" s="143"/>
+      <c r="B12" s="133"/>
+      <c r="C12" s="133"/>
+      <c r="D12" s="133"/>
+      <c r="E12" s="133"/>
       <c r="F12" s="63">
         <v>0</v>
       </c>
-      <c r="H12" s="144" t="str">
+      <c r="H12" s="124" t="str">
         <f>CONCATENATE((N8+F12+F13+F14+F15+F11)/20, " meses")</f>
-        <v>1.1 meses</v>
-      </c>
-      <c r="I12" s="144"/>
-      <c r="J12" s="144"/>
+        <v>0.325 meses</v>
+      </c>
+      <c r="I12" s="124"/>
+      <c r="J12" s="124"/>
     </row>
     <row r="13" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="143" t="s">
+      <c r="A13" s="133" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="143"/>
-      <c r="C13" s="143"/>
-      <c r="D13" s="143"/>
-      <c r="E13" s="143"/>
+      <c r="B13" s="133"/>
+      <c r="C13" s="133"/>
+      <c r="D13" s="133"/>
+      <c r="E13" s="133"/>
       <c r="F13" s="63">
         <v>1</v>
       </c>
-      <c r="H13" s="145">
+      <c r="H13" s="125">
         <f>((N8+F12+F13+F14+F15+F11)/20)</f>
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="I13" s="145"/>
-      <c r="J13" s="145"/>
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="I13" s="125"/>
+      <c r="J13" s="125"/>
       <c r="K13" s="65" t="s">
         <v>46</v>
       </c>
       <c r="L13" s="65"/>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A14" s="143" t="s">
+      <c r="A14" s="133" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="143"/>
-      <c r="C14" s="143"/>
-      <c r="D14" s="143"/>
-      <c r="E14" s="143"/>
+      <c r="B14" s="133"/>
+      <c r="C14" s="133"/>
+      <c r="D14" s="133"/>
+      <c r="E14" s="133"/>
       <c r="F14" s="63">
         <v>0.5</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A15" s="143" t="s">
+      <c r="A15" s="133" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="143"/>
-      <c r="C15" s="143"/>
-      <c r="D15" s="143"/>
-      <c r="E15" s="143"/>
+      <c r="B15" s="133"/>
+      <c r="C15" s="133"/>
+      <c r="D15" s="133"/>
+      <c r="E15" s="133"/>
       <c r="F15" s="63">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.2">
@@ -2897,271 +2923,271 @@
       <c r="F21" s="9"/>
     </row>
     <row r="22" spans="1:21" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="H22" s="128" t="s">
+      <c r="H22" s="149" t="s">
         <v>164</v>
       </c>
-      <c r="I22" s="128"/>
-      <c r="J22" s="128"/>
-      <c r="K22" s="128"/>
-      <c r="L22" s="128"/>
-      <c r="M22" s="128"/>
-      <c r="N22" s="128"/>
-      <c r="O22" s="128"/>
-      <c r="P22" s="128"/>
-      <c r="Q22" s="128"/>
-      <c r="R22" s="128"/>
-      <c r="S22" s="128"/>
-      <c r="T22" s="128"/>
-      <c r="U22" s="128"/>
+      <c r="I22" s="149"/>
+      <c r="J22" s="149"/>
+      <c r="K22" s="149"/>
+      <c r="L22" s="149"/>
+      <c r="M22" s="149"/>
+      <c r="N22" s="149"/>
+      <c r="O22" s="149"/>
+      <c r="P22" s="149"/>
+      <c r="Q22" s="149"/>
+      <c r="R22" s="149"/>
+      <c r="S22" s="149"/>
+      <c r="T22" s="149"/>
+      <c r="U22" s="149"/>
     </row>
     <row r="23" spans="1:21" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="134" t="s">
+      <c r="A23" s="139" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="135"/>
-      <c r="C23" s="135"/>
-      <c r="D23" s="135"/>
-      <c r="E23" s="135"/>
-      <c r="F23" s="136"/>
-      <c r="H23" s="125" t="s">
+      <c r="B23" s="140"/>
+      <c r="C23" s="140"/>
+      <c r="D23" s="140"/>
+      <c r="E23" s="140"/>
+      <c r="F23" s="141"/>
+      <c r="H23" s="151" t="s">
         <v>165</v>
       </c>
-      <c r="I23" s="125"/>
-      <c r="J23" s="125"/>
-      <c r="K23" s="125"/>
-      <c r="L23" s="125" t="s">
+      <c r="I23" s="151"/>
+      <c r="J23" s="151"/>
+      <c r="K23" s="151"/>
+      <c r="L23" s="151" t="s">
         <v>166</v>
       </c>
-      <c r="M23" s="125"/>
-      <c r="N23" s="125"/>
-      <c r="O23" s="125"/>
-      <c r="P23" s="125"/>
-      <c r="Q23" s="125"/>
-      <c r="R23" s="125"/>
-      <c r="S23" s="125"/>
-      <c r="T23" s="125"/>
-      <c r="U23" s="125"/>
+      <c r="M23" s="151"/>
+      <c r="N23" s="151"/>
+      <c r="O23" s="151"/>
+      <c r="P23" s="151"/>
+      <c r="Q23" s="151"/>
+      <c r="R23" s="151"/>
+      <c r="S23" s="151"/>
+      <c r="T23" s="151"/>
+      <c r="U23" s="151"/>
     </row>
     <row r="24" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="137" t="s">
+      <c r="A24" s="142" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="138"/>
-      <c r="C24" s="138"/>
-      <c r="D24" s="138"/>
-      <c r="E24" s="138"/>
+      <c r="B24" s="143"/>
+      <c r="C24" s="143"/>
+      <c r="D24" s="143"/>
+      <c r="E24" s="143"/>
       <c r="F24" s="82">
         <f>F11</f>
         <v>0.5</v>
       </c>
-      <c r="H24" s="129" t="str">
+      <c r="H24" s="134" t="str">
         <f>A24</f>
         <v>Preparación de equipo y ambientes</v>
       </c>
-      <c r="I24" s="129"/>
-      <c r="J24" s="129"/>
-      <c r="K24" s="129"/>
-      <c r="L24" s="127"/>
-      <c r="M24" s="127"/>
-      <c r="N24" s="127"/>
-      <c r="O24" s="127"/>
-      <c r="P24" s="127"/>
-      <c r="Q24" s="127"/>
-      <c r="R24" s="127"/>
-      <c r="S24" s="127"/>
-      <c r="T24" s="127"/>
-      <c r="U24" s="127"/>
+      <c r="I24" s="134"/>
+      <c r="J24" s="134"/>
+      <c r="K24" s="134"/>
+      <c r="L24" s="148"/>
+      <c r="M24" s="148"/>
+      <c r="N24" s="148"/>
+      <c r="O24" s="148"/>
+      <c r="P24" s="148"/>
+      <c r="Q24" s="148"/>
+      <c r="R24" s="148"/>
+      <c r="S24" s="148"/>
+      <c r="T24" s="148"/>
+      <c r="U24" s="148"/>
     </row>
     <row r="25" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="137" t="s">
+      <c r="A25" s="142" t="s">
         <v>55</v>
       </c>
-      <c r="B25" s="138"/>
-      <c r="C25" s="138"/>
-      <c r="D25" s="138"/>
-      <c r="E25" s="138"/>
+      <c r="B25" s="143"/>
+      <c r="C25" s="143"/>
+      <c r="D25" s="143"/>
+      <c r="E25" s="143"/>
       <c r="F25" s="82">
         <f>F12</f>
         <v>0</v>
       </c>
-      <c r="H25" s="129" t="str">
+      <c r="H25" s="134" t="str">
         <f t="shared" ref="H25:H29" si="0">A25</f>
         <v>Exploración del negocio</v>
       </c>
-      <c r="I25" s="129"/>
-      <c r="J25" s="129"/>
-      <c r="K25" s="129"/>
-      <c r="L25" s="127"/>
-      <c r="M25" s="127"/>
-      <c r="N25" s="127"/>
-      <c r="O25" s="127"/>
-      <c r="P25" s="127"/>
-      <c r="Q25" s="127"/>
-      <c r="R25" s="127"/>
-      <c r="S25" s="127"/>
-      <c r="T25" s="127"/>
-      <c r="U25" s="127"/>
+      <c r="I25" s="134"/>
+      <c r="J25" s="134"/>
+      <c r="K25" s="134"/>
+      <c r="L25" s="148"/>
+      <c r="M25" s="148"/>
+      <c r="N25" s="148"/>
+      <c r="O25" s="148"/>
+      <c r="P25" s="148"/>
+      <c r="Q25" s="148"/>
+      <c r="R25" s="148"/>
+      <c r="S25" s="148"/>
+      <c r="T25" s="148"/>
+      <c r="U25" s="148"/>
     </row>
     <row r="26" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="139" t="str">
+      <c r="A26" s="144" t="str">
         <f>CONCATENATE("Desarrollo del sistema - (",F7,") Iteraci",IF(F7&gt;1,"ones","ón"))</f>
         <v>Desarrollo del sistema - (1) Iteración</v>
       </c>
-      <c r="B26" s="140"/>
-      <c r="C26" s="140"/>
-      <c r="D26" s="140"/>
-      <c r="E26" s="140"/>
+      <c r="B26" s="145"/>
+      <c r="C26" s="145"/>
+      <c r="D26" s="145"/>
+      <c r="E26" s="145"/>
       <c r="F26" s="83">
         <f>N8</f>
-        <v>19</v>
-      </c>
-      <c r="H26" s="129" t="str">
+        <v>4</v>
+      </c>
+      <c r="H26" s="134" t="str">
         <f t="shared" si="0"/>
         <v>Desarrollo del sistema - (1) Iteración</v>
       </c>
-      <c r="I26" s="129"/>
-      <c r="J26" s="129"/>
-      <c r="K26" s="129"/>
-      <c r="L26" s="127"/>
-      <c r="M26" s="127"/>
-      <c r="N26" s="127"/>
-      <c r="O26" s="127"/>
-      <c r="P26" s="127"/>
-      <c r="Q26" s="127"/>
-      <c r="R26" s="127"/>
-      <c r="S26" s="127"/>
-      <c r="T26" s="127"/>
-      <c r="U26" s="127"/>
+      <c r="I26" s="134"/>
+      <c r="J26" s="134"/>
+      <c r="K26" s="134"/>
+      <c r="L26" s="148"/>
+      <c r="M26" s="148"/>
+      <c r="N26" s="148"/>
+      <c r="O26" s="148"/>
+      <c r="P26" s="148"/>
+      <c r="Q26" s="148"/>
+      <c r="R26" s="148"/>
+      <c r="S26" s="148"/>
+      <c r="T26" s="148"/>
+      <c r="U26" s="148"/>
     </row>
     <row r="27" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="139" t="s">
+      <c r="A27" s="144" t="s">
         <v>56</v>
       </c>
-      <c r="B27" s="140"/>
-      <c r="C27" s="140"/>
-      <c r="D27" s="140"/>
-      <c r="E27" s="140"/>
+      <c r="B27" s="145"/>
+      <c r="C27" s="145"/>
+      <c r="D27" s="145"/>
+      <c r="E27" s="145"/>
       <c r="F27" s="83">
         <f>F13</f>
         <v>1</v>
       </c>
-      <c r="H27" s="129" t="str">
+      <c r="H27" s="134" t="str">
         <f t="shared" si="0"/>
         <v>Documentación, pruebas integrales y estabilización</v>
       </c>
-      <c r="I27" s="129"/>
-      <c r="J27" s="129"/>
-      <c r="K27" s="129"/>
-      <c r="L27" s="127"/>
-      <c r="M27" s="127"/>
-      <c r="N27" s="127"/>
-      <c r="O27" s="127"/>
-      <c r="P27" s="127"/>
-      <c r="Q27" s="127"/>
-      <c r="R27" s="127"/>
-      <c r="S27" s="127"/>
-      <c r="T27" s="127"/>
-      <c r="U27" s="127"/>
+      <c r="I27" s="134"/>
+      <c r="J27" s="134"/>
+      <c r="K27" s="134"/>
+      <c r="L27" s="148"/>
+      <c r="M27" s="148"/>
+      <c r="N27" s="148"/>
+      <c r="O27" s="148"/>
+      <c r="P27" s="148"/>
+      <c r="Q27" s="148"/>
+      <c r="R27" s="148"/>
+      <c r="S27" s="148"/>
+      <c r="T27" s="148"/>
+      <c r="U27" s="148"/>
     </row>
     <row r="28" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="139" t="s">
+      <c r="A28" s="144" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="140"/>
-      <c r="C28" s="140"/>
-      <c r="D28" s="140"/>
-      <c r="E28" s="140"/>
+      <c r="B28" s="145"/>
+      <c r="C28" s="145"/>
+      <c r="D28" s="145"/>
+      <c r="E28" s="145"/>
       <c r="F28" s="83">
         <f>F14</f>
         <v>0.5</v>
       </c>
-      <c r="H28" s="129" t="str">
+      <c r="H28" s="134" t="str">
         <f t="shared" si="0"/>
         <v>Instalación</v>
       </c>
-      <c r="I28" s="129"/>
-      <c r="J28" s="129"/>
-      <c r="K28" s="129"/>
-      <c r="L28" s="127"/>
-      <c r="M28" s="127"/>
-      <c r="N28" s="127"/>
-      <c r="O28" s="127"/>
-      <c r="P28" s="127"/>
-      <c r="Q28" s="127"/>
-      <c r="R28" s="127"/>
-      <c r="S28" s="127"/>
-      <c r="T28" s="127"/>
-      <c r="U28" s="127"/>
+      <c r="I28" s="134"/>
+      <c r="J28" s="134"/>
+      <c r="K28" s="134"/>
+      <c r="L28" s="148"/>
+      <c r="M28" s="148"/>
+      <c r="N28" s="148"/>
+      <c r="O28" s="148"/>
+      <c r="P28" s="148"/>
+      <c r="Q28" s="148"/>
+      <c r="R28" s="148"/>
+      <c r="S28" s="148"/>
+      <c r="T28" s="148"/>
+      <c r="U28" s="148"/>
     </row>
     <row r="29" spans="1:21" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="141" t="s">
+      <c r="A29" s="146" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="142"/>
-      <c r="C29" s="142"/>
-      <c r="D29" s="142"/>
-      <c r="E29" s="142"/>
+      <c r="B29" s="147"/>
+      <c r="C29" s="147"/>
+      <c r="D29" s="147"/>
+      <c r="E29" s="147"/>
       <c r="F29" s="84">
         <f>F15</f>
-        <v>1</v>
-      </c>
-      <c r="H29" s="129" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="H29" s="134" t="str">
         <f t="shared" si="0"/>
         <v>Acompañamiento en producción</v>
       </c>
-      <c r="I29" s="129"/>
-      <c r="J29" s="129"/>
-      <c r="K29" s="129"/>
-      <c r="L29" s="127"/>
-      <c r="M29" s="127"/>
-      <c r="N29" s="127"/>
-      <c r="O29" s="127"/>
-      <c r="P29" s="127"/>
-      <c r="Q29" s="127"/>
-      <c r="R29" s="127"/>
-      <c r="S29" s="127"/>
-      <c r="T29" s="127"/>
-      <c r="U29" s="127"/>
+      <c r="I29" s="134"/>
+      <c r="J29" s="134"/>
+      <c r="K29" s="134"/>
+      <c r="L29" s="148"/>
+      <c r="M29" s="148"/>
+      <c r="N29" s="148"/>
+      <c r="O29" s="148"/>
+      <c r="P29" s="148"/>
+      <c r="Q29" s="148"/>
+      <c r="R29" s="148"/>
+      <c r="S29" s="148"/>
+      <c r="T29" s="148"/>
+      <c r="U29" s="148"/>
     </row>
     <row r="30" spans="1:21" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A30" s="130" t="s">
+      <c r="A30" s="135" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="131"/>
-      <c r="C30" s="131"/>
-      <c r="D30" s="131"/>
-      <c r="E30" s="131"/>
+      <c r="B30" s="136"/>
+      <c r="C30" s="136"/>
+      <c r="D30" s="136"/>
+      <c r="E30" s="136"/>
       <c r="F30" s="85">
         <f>SUM(F24:F29)</f>
-        <v>22</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="31" spans="1:21" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="132" t="s">
+      <c r="A31" s="137" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="133"/>
-      <c r="C31" s="133"/>
-      <c r="D31" s="133"/>
-      <c r="E31" s="133"/>
+      <c r="B31" s="138"/>
+      <c r="C31" s="138"/>
+      <c r="D31" s="138"/>
+      <c r="E31" s="138"/>
       <c r="F31" s="86">
         <f>F30/20</f>
-        <v>1.1000000000000001</v>
+        <v>0.32500000000000001</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="H32" s="126" t="s">
+      <c r="H32" s="152" t="s">
         <v>172</v>
       </c>
-      <c r="I32" s="126"/>
-      <c r="J32" s="126"/>
-      <c r="K32" s="126"/>
-      <c r="L32" s="126"/>
-      <c r="M32" s="126"/>
-      <c r="N32" s="126"/>
-      <c r="O32" s="126"/>
-      <c r="P32" s="126"/>
-      <c r="Q32" s="126"/>
+      <c r="I32" s="152"/>
+      <c r="J32" s="152"/>
+      <c r="K32" s="152"/>
+      <c r="L32" s="152"/>
+      <c r="M32" s="152"/>
+      <c r="N32" s="152"/>
+      <c r="O32" s="152"/>
+      <c r="P32" s="152"/>
+      <c r="Q32" s="152"/>
     </row>
     <row r="33" spans="8:17" x14ac:dyDescent="0.2">
       <c r="H33" s="114" t="s">
@@ -3173,157 +3199,137 @@
       <c r="J33" s="114" t="s">
         <v>111</v>
       </c>
-      <c r="K33" s="125" t="s">
+      <c r="K33" s="151" t="s">
         <v>169</v>
       </c>
-      <c r="L33" s="125"/>
-      <c r="M33" s="125"/>
-      <c r="N33" s="125"/>
-      <c r="O33" s="125"/>
-      <c r="P33" s="125"/>
-      <c r="Q33" s="125"/>
+      <c r="L33" s="151"/>
+      <c r="M33" s="151"/>
+      <c r="N33" s="151"/>
+      <c r="O33" s="151"/>
+      <c r="P33" s="151"/>
+      <c r="Q33" s="151"/>
     </row>
     <row r="34" spans="8:17" x14ac:dyDescent="0.2">
       <c r="H34" s="115"/>
       <c r="I34" s="115"/>
       <c r="J34" s="115"/>
-      <c r="K34" s="124"/>
-      <c r="L34" s="124"/>
-      <c r="M34" s="124"/>
-      <c r="N34" s="124"/>
-      <c r="O34" s="124"/>
-      <c r="P34" s="124"/>
-      <c r="Q34" s="124"/>
+      <c r="K34" s="150"/>
+      <c r="L34" s="150"/>
+      <c r="M34" s="150"/>
+      <c r="N34" s="150"/>
+      <c r="O34" s="150"/>
+      <c r="P34" s="150"/>
+      <c r="Q34" s="150"/>
     </row>
     <row r="35" spans="8:17" x14ac:dyDescent="0.2">
       <c r="H35" s="115"/>
       <c r="I35" s="115"/>
       <c r="J35" s="115"/>
-      <c r="K35" s="124"/>
-      <c r="L35" s="124"/>
-      <c r="M35" s="124"/>
-      <c r="N35" s="124"/>
-      <c r="O35" s="124"/>
-      <c r="P35" s="124"/>
-      <c r="Q35" s="124"/>
+      <c r="K35" s="150"/>
+      <c r="L35" s="150"/>
+      <c r="M35" s="150"/>
+      <c r="N35" s="150"/>
+      <c r="O35" s="150"/>
+      <c r="P35" s="150"/>
+      <c r="Q35" s="150"/>
     </row>
     <row r="36" spans="8:17" x14ac:dyDescent="0.2">
       <c r="H36" s="115"/>
       <c r="I36" s="115"/>
       <c r="J36" s="115"/>
-      <c r="K36" s="124"/>
-      <c r="L36" s="124"/>
-      <c r="M36" s="124"/>
-      <c r="N36" s="124"/>
-      <c r="O36" s="124"/>
-      <c r="P36" s="124"/>
-      <c r="Q36" s="124"/>
+      <c r="K36" s="150"/>
+      <c r="L36" s="150"/>
+      <c r="M36" s="150"/>
+      <c r="N36" s="150"/>
+      <c r="O36" s="150"/>
+      <c r="P36" s="150"/>
+      <c r="Q36" s="150"/>
     </row>
     <row r="37" spans="8:17" x14ac:dyDescent="0.2">
       <c r="H37" s="115"/>
       <c r="I37" s="115"/>
       <c r="J37" s="115"/>
-      <c r="K37" s="124"/>
-      <c r="L37" s="124"/>
-      <c r="M37" s="124"/>
-      <c r="N37" s="124"/>
-      <c r="O37" s="124"/>
-      <c r="P37" s="124"/>
-      <c r="Q37" s="124"/>
+      <c r="K37" s="150"/>
+      <c r="L37" s="150"/>
+      <c r="M37" s="150"/>
+      <c r="N37" s="150"/>
+      <c r="O37" s="150"/>
+      <c r="P37" s="150"/>
+      <c r="Q37" s="150"/>
     </row>
     <row r="38" spans="8:17" x14ac:dyDescent="0.2">
       <c r="H38" s="115"/>
       <c r="I38" s="115"/>
       <c r="J38" s="115"/>
-      <c r="K38" s="124"/>
-      <c r="L38" s="124"/>
-      <c r="M38" s="124"/>
-      <c r="N38" s="124"/>
-      <c r="O38" s="124"/>
-      <c r="P38" s="124"/>
-      <c r="Q38" s="124"/>
+      <c r="K38" s="150"/>
+      <c r="L38" s="150"/>
+      <c r="M38" s="150"/>
+      <c r="N38" s="150"/>
+      <c r="O38" s="150"/>
+      <c r="P38" s="150"/>
+      <c r="Q38" s="150"/>
     </row>
     <row r="39" spans="8:17" x14ac:dyDescent="0.2">
       <c r="H39" s="115"/>
       <c r="I39" s="115"/>
       <c r="J39" s="115"/>
-      <c r="K39" s="124"/>
-      <c r="L39" s="124"/>
-      <c r="M39" s="124"/>
-      <c r="N39" s="124"/>
-      <c r="O39" s="124"/>
-      <c r="P39" s="124"/>
-      <c r="Q39" s="124"/>
+      <c r="K39" s="150"/>
+      <c r="L39" s="150"/>
+      <c r="M39" s="150"/>
+      <c r="N39" s="150"/>
+      <c r="O39" s="150"/>
+      <c r="P39" s="150"/>
+      <c r="Q39" s="150"/>
     </row>
     <row r="40" spans="8:17" x14ac:dyDescent="0.2">
       <c r="H40" s="115"/>
       <c r="I40" s="115"/>
       <c r="J40" s="115"/>
-      <c r="K40" s="124"/>
-      <c r="L40" s="124"/>
-      <c r="M40" s="124"/>
-      <c r="N40" s="124"/>
-      <c r="O40" s="124"/>
-      <c r="P40" s="124"/>
-      <c r="Q40" s="124"/>
+      <c r="K40" s="150"/>
+      <c r="L40" s="150"/>
+      <c r="M40" s="150"/>
+      <c r="N40" s="150"/>
+      <c r="O40" s="150"/>
+      <c r="P40" s="150"/>
+      <c r="Q40" s="150"/>
     </row>
     <row r="41" spans="8:17" x14ac:dyDescent="0.2">
       <c r="H41" s="115"/>
       <c r="I41" s="115"/>
       <c r="J41" s="115"/>
-      <c r="K41" s="124"/>
-      <c r="L41" s="124"/>
-      <c r="M41" s="124"/>
-      <c r="N41" s="124"/>
-      <c r="O41" s="124"/>
-      <c r="P41" s="124"/>
-      <c r="Q41" s="124"/>
+      <c r="K41" s="150"/>
+      <c r="L41" s="150"/>
+      <c r="M41" s="150"/>
+      <c r="N41" s="150"/>
+      <c r="O41" s="150"/>
+      <c r="P41" s="150"/>
+      <c r="Q41" s="150"/>
     </row>
     <row r="42" spans="8:17" x14ac:dyDescent="0.2">
       <c r="H42" s="115"/>
       <c r="I42" s="115"/>
       <c r="J42" s="115"/>
-      <c r="K42" s="124"/>
-      <c r="L42" s="124"/>
-      <c r="M42" s="124"/>
-      <c r="N42" s="124"/>
-      <c r="O42" s="124"/>
-      <c r="P42" s="124"/>
-      <c r="Q42" s="124"/>
+      <c r="K42" s="150"/>
+      <c r="L42" s="150"/>
+      <c r="M42" s="150"/>
+      <c r="N42" s="150"/>
+      <c r="O42" s="150"/>
+      <c r="P42" s="150"/>
+      <c r="Q42" s="150"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <mergeCells count="55">
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="H3:M3"/>
-    <mergeCell ref="H4:M4"/>
-    <mergeCell ref="H5:M5"/>
-    <mergeCell ref="H6:M6"/>
-    <mergeCell ref="H7:M7"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="H27:K27"/>
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A31:E31"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A24:E24"/>
+  <mergeCells count="57">
+    <mergeCell ref="P2:Q3"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="K41:Q41"/>
+    <mergeCell ref="K42:Q42"/>
+    <mergeCell ref="K33:Q33"/>
+    <mergeCell ref="H32:Q32"/>
+    <mergeCell ref="K36:Q36"/>
+    <mergeCell ref="K37:Q37"/>
+    <mergeCell ref="K38:Q38"/>
+    <mergeCell ref="K39:Q39"/>
+    <mergeCell ref="K40:Q40"/>
     <mergeCell ref="L28:U28"/>
     <mergeCell ref="L29:U29"/>
     <mergeCell ref="H22:U22"/>
@@ -3340,17 +3346,38 @@
     <mergeCell ref="H24:K24"/>
     <mergeCell ref="H25:K25"/>
     <mergeCell ref="H26:K26"/>
-    <mergeCell ref="K41:Q41"/>
-    <mergeCell ref="K42:Q42"/>
-    <mergeCell ref="K33:Q33"/>
-    <mergeCell ref="H32:Q32"/>
-    <mergeCell ref="K36:Q36"/>
-    <mergeCell ref="K37:Q37"/>
-    <mergeCell ref="K38:Q38"/>
-    <mergeCell ref="K39:Q39"/>
-    <mergeCell ref="K40:Q40"/>
+    <mergeCell ref="H27:K27"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A7:E7"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H3:M3"/>
+    <mergeCell ref="H4:M4"/>
+    <mergeCell ref="H5:M5"/>
+    <mergeCell ref="H6:M6"/>
+    <mergeCell ref="H7:M7"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I34:J42">
       <formula1>$AA$1:$AA$2</formula1>
     </dataValidation>
@@ -3437,14 +3464,14 @@
       </c>
       <c r="B2" s="12">
         <f>+C5+C8+C11+C14+C17+C20+C23+C29+C26+C32+C35+C38+C41+C44+C47</f>
-        <v>10900000</v>
+        <v>2198863.6363636362</v>
       </c>
       <c r="C2" s="106" t="s">
         <v>80</v>
       </c>
       <c r="D2" s="1">
         <f>+D5+D8+D11+D14+D17+D20+D23+D29+D26+D32+D35+D38+D41+D44+D47</f>
-        <v>10900000</v>
+        <v>2198863.6363636362</v>
       </c>
       <c r="E2" s="1">
         <f t="shared" ref="E2:U2" si="0">+E5+E8+E11+E14+E17+E20+E23+E29+E26+E32+E35+E38+E41+E44+E47</f>
@@ -3550,10 +3577,10 @@
       </c>
       <c r="C4" s="2">
         <f>SUM(D4:U4)</f>
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="D4" s="60">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="E4" s="60"/>
       <c r="F4" s="60"/>
@@ -3576,11 +3603,11 @@
     <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C5" s="3">
         <f>SUM(D5:U5)</f>
-        <v>3000000</v>
+        <v>460227.27272727276</v>
       </c>
       <c r="D5" s="1">
-        <f>D4*D3</f>
-        <v>3000000</v>
+        <f>(D4*D3)*((Iteraciones!$P$4)/22)</f>
+        <v>460227.27272727276</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" ref="E5:M5" si="1">E4*E3</f>
@@ -3686,10 +3713,10 @@
       </c>
       <c r="C7" s="2">
         <f>SUM(D7:U7)</f>
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="D7" s="60">
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="E7" s="60"/>
       <c r="F7" s="60"/>
@@ -3712,11 +3739,11 @@
     <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C8" s="3">
         <f>SUM(D8:U8)</f>
-        <v>7200000</v>
+        <v>1595454.5454545456</v>
       </c>
       <c r="D8" s="1">
-        <f>D7*D6</f>
-        <v>7200000</v>
+        <f>(D7*D6)*((Iteraciones!$P$4)/22)</f>
+        <v>1595454.5454545456</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" ref="E8" si="4">E7*E6</f>
@@ -3848,11 +3875,11 @@
     <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C11" s="3">
         <f>SUM(D11:U11)</f>
-        <v>300000</v>
+        <v>61363.636363636368</v>
       </c>
       <c r="D11" s="1">
-        <f>D10*D9</f>
-        <v>300000</v>
+        <f>(D10*D9)*((Iteraciones!$P$4)/22)</f>
+        <v>61363.636363636368</v>
       </c>
       <c r="E11" s="1">
         <f t="shared" ref="E11" si="14">E10*E9</f>
@@ -3984,11 +4011,11 @@
     <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C14" s="3">
         <f>SUM(D14:U14)</f>
-        <v>400000</v>
+        <v>81818.181818181823</v>
       </c>
       <c r="D14" s="1">
-        <f>D13*D12</f>
-        <v>400000</v>
+        <f>(D13*D12)*((Iteraciones!$P$4)/22)</f>
+        <v>81818.181818181823</v>
       </c>
       <c r="E14" s="1">
         <f t="shared" ref="E14" si="24">E13*E12</f>
@@ -5842,7 +5869,7 @@
       </c>
       <c r="B60" s="153">
         <f>CEILING(B50+B2,100000)</f>
-        <v>10900000</v>
+        <v>2200000</v>
       </c>
       <c r="C60" s="154"/>
     </row>
@@ -5862,7 +5889,7 @@
       </c>
       <c r="C62" s="47">
         <f>$B$60*B62</f>
-        <v>1199000</v>
+        <v>242000</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.2">
@@ -5903,7 +5930,7 @@
       </c>
       <c r="B66" s="155">
         <f>CEILING(+B60+C64+B61+C62+C63+C65,100000)</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="C66" s="156"/>
     </row>
@@ -5926,7 +5953,7 @@
       </c>
       <c r="D69" s="19">
         <f>SUM(D70:D77)*$B$66</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="E69" s="19">
         <f t="shared" ref="E69:M69" si="56">SUM(E70:E77)*$B$66</f>
@@ -6007,7 +6034,7 @@
       </c>
       <c r="C70" s="81">
         <f>SUM(D70:U70)*$B$66</f>
-        <v>4840000</v>
+        <v>1000000</v>
       </c>
       <c r="D70" s="60">
         <v>0.4</v>
@@ -6040,7 +6067,7 @@
       </c>
       <c r="C71" s="81">
         <f t="shared" ref="C71:C77" si="61">SUM(D71:U71)*$B$66</f>
-        <v>7260000</v>
+        <v>1500000</v>
       </c>
       <c r="D71" s="60">
         <v>0.6</v>
@@ -6259,7 +6286,7 @@
       </c>
       <c r="C78" s="74">
         <f t="shared" si="62"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.2">
@@ -6268,7 +6295,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="3">
     <mergeCell ref="B60:C60"/>
     <mergeCell ref="B66:C66"/>
@@ -6521,11 +6547,11 @@
       </c>
       <c r="C4" s="2">
         <f>SUM(D4:U4)</f>
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="D4" s="60">
         <f>'A cobrar'!D4</f>
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="E4" s="60">
         <f>'A cobrar'!E4</f>
@@ -6762,11 +6788,11 @@
       </c>
       <c r="C7" s="2">
         <f>SUM(D7:U7)</f>
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="D7" s="60">
         <f>'A cobrar'!D7</f>
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="E7" s="60">
         <f>'A cobrar'!E7</f>
@@ -10913,7 +10939,7 @@
       </c>
       <c r="B64" s="41">
         <f>'A cobrar'!B66:C66*(0.00966+0.008)</f>
-        <v>213686.00000000003</v>
+        <v>44150.000000000007</v>
       </c>
       <c r="C64" s="42"/>
       <c r="D64" s="43">
@@ -10995,7 +11021,7 @@
       </c>
       <c r="B65" s="41">
         <f>'A cobrar'!B66:C66*0.004</f>
-        <v>48400</v>
+        <v>10000</v>
       </c>
       <c r="C65" s="42"/>
       <c r="D65" s="43">
@@ -11113,7 +11139,7 @@
       </c>
       <c r="B68" s="53">
         <f>B61+B64+B65</f>
-        <v>262086.00000000003</v>
+        <v>54150.000000000007</v>
       </c>
       <c r="C68" s="33"/>
       <c r="D68" s="34">
@@ -14475,7 +14501,7 @@
       </c>
       <c r="D2" s="91">
         <f>'A cobrar'!D69-'Costos planeados'!D68</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="E2" s="91">
         <f>'A cobrar'!E69-'Costos planeados'!E68</f>
@@ -14552,75 +14578,75 @@
       </c>
       <c r="D3" s="92">
         <f>D2</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="E3" s="92">
         <f t="shared" ref="E3:O3" si="0">D3+E2</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="F3" s="92">
         <f t="shared" si="0"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="G3" s="92">
         <f t="shared" si="0"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="H3" s="92">
         <f t="shared" si="0"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="I3" s="92">
         <f t="shared" si="0"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="J3" s="92">
         <f t="shared" si="0"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="K3" s="92">
         <f t="shared" si="0"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="L3" s="92">
         <f t="shared" si="0"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="M3" s="92">
         <f t="shared" si="0"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="N3" s="92">
         <f t="shared" si="0"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="O3" s="92">
         <f t="shared" si="0"/>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="P3" s="92">
         <f t="shared" ref="P3" si="1">O3+P2</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="Q3" s="92">
         <f t="shared" ref="Q3" si="2">P3+Q2</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="R3" s="92">
         <f t="shared" ref="R3" si="3">Q3+R2</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="S3" s="92">
         <f t="shared" ref="S3" si="4">R3+S2</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="T3" s="92">
         <f t="shared" ref="T3" si="5">S3+T2</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="U3" s="92">
         <f t="shared" ref="U3" si="6">T3+U2</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.2">
@@ -14629,7 +14655,7 @@
       </c>
       <c r="B4" s="91">
         <f>'A cobrar'!B66:C66</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.2">
@@ -14638,7 +14664,7 @@
       </c>
       <c r="B5" s="91">
         <f>'Costos planeados'!B68</f>
-        <v>262086.00000000003</v>
+        <v>54150.000000000007</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.2">
@@ -14656,7 +14682,7 @@
       </c>
       <c r="B7" s="91">
         <f>B4-B5-B6</f>
-        <v>11837914</v>
+        <v>2445850</v>
       </c>
       <c r="D7" s="51" t="str">
         <f>IF(B7&lt;0,"Este proyecto dá perdida!!!","")</f>
@@ -14907,7 +14933,7 @@
       </c>
       <c r="B4" s="91">
         <f>'A cobrar'!B66:C66</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.2">
@@ -14934,7 +14960,7 @@
       </c>
       <c r="B7" s="91">
         <f>B4-B5-B6</f>
-        <v>12100000</v>
+        <v>2500000</v>
       </c>
       <c r="D7" s="51" t="str">
         <f>IF(B7&lt;0,"Este proyecto dá perdida!!!","")</f>
@@ -14965,7 +14991,7 @@
     <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D13" s="94">
         <f>D2-'Caja planeada'!D2</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="E13" s="94">
         <f>E2-'Caja planeada'!E2</f>
@@ -15044,75 +15070,75 @@
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="D16" s="94">
         <f>D3-'Caja planeada'!D3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="E16" s="94">
         <f>E3-'Caja planeada'!E3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="F16" s="94">
         <f>F3-'Caja planeada'!F3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="G16" s="94">
         <f>G3-'Caja planeada'!G3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="H16" s="94">
         <f>H3-'Caja planeada'!H3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="I16" s="94">
         <f>I3-'Caja planeada'!I3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="J16" s="94">
         <f>J3-'Caja planeada'!J3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="K16" s="94">
         <f>K3-'Caja planeada'!K3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="L16" s="94">
         <f>L3-'Caja planeada'!L3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="M16" s="94">
         <f>M3-'Caja planeada'!M3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="N16" s="94">
         <f>N3-'Caja planeada'!N3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="O16" s="94">
         <f>O3-'Caja planeada'!O3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="P16" s="94">
         <f>P3-'Caja planeada'!P3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="Q16" s="94">
         <f>Q3-'Caja planeada'!Q3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="R16" s="94">
         <f>R3-'Caja planeada'!R3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="S16" s="94">
         <f>S3-'Caja planeada'!S3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="T16" s="94">
         <f>T3-'Caja planeada'!T3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
       <c r="U16" s="94">
         <f>U3-'Caja planeada'!U3</f>
-        <v>-12100000</v>
+        <v>-2500000</v>
       </c>
     </row>
   </sheetData>
@@ -15137,28 +15163,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <SharedWithUsers xmlns="ceb8ebac-74c3-43a7-a348-c9253525119c">
-      <UserInfo>
-        <DisplayName>Liliana Constanza  Silva Yepes</DisplayName>
-        <AccountId>650</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Julieth Paola Quintero</DisplayName>
-        <AccountId>19</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="ceb8ebac-74c3-43a7-a348-c9253525119c" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="429a2966-0d94-4baf-ac31-c583b7569082">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -15428,28 +15438,34 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <SharedWithUsers xmlns="ceb8ebac-74c3-43a7-a348-c9253525119c">
+      <UserInfo>
+        <DisplayName>Liliana Constanza  Silva Yepes</DisplayName>
+        <AccountId>650</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Julieth Paola Quintero</DisplayName>
+        <AccountId>19</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="ceb8ebac-74c3-43a7-a348-c9253525119c" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="429a2966-0d94-4baf-ac31-c583b7569082">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87525ABF-8997-49A0-9C96-F6ADAC240FC0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04C3FD96-9D8A-4970-967D-E9957C77AF54}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="ceb8ebac-74c3-43a7-a348-c9253525119c"/>
-    <ds:schemaRef ds:uri="429a2966-0d94-4baf-ac31-c583b7569082"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -15475,9 +15491,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04C3FD96-9D8A-4970-967D-E9957C77AF54}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87525ABF-8997-49A0-9C96-F6ADAC240FC0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="ceb8ebac-74c3-43a7-a348-c9253525119c"/>
+    <ds:schemaRef ds:uri="429a2966-0d94-4baf-ac31-c583b7569082"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>